<commit_message>
feat: improve bilingual Excel import template
</commit_message>
<xml_diff>
--- a/Good Conduct Data Template.xlsx
+++ b/Good Conduct Data Template.xlsx
@@ -5,6 +5,7 @@
   <sheets>
     <sheet name="Good Conduct" sheetId="1" r:id="rId1"/>
     <sheet name="Instructions" sheetId="2" r:id="rId2"/>
+    <sheet name="Field Guide" sheetId="3" r:id="rId3"/>
   </sheets>
 </workbook>
 </file>
@@ -398,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB2"/>
+  <dimension ref="A1:AD2"/>
   <cols>
     <col min="1" max="1" width="22.83203125" customWidth="1"/>
     <col min="2" max="2" width="22.83203125" customWidth="1"/>
@@ -428,190 +429,204 @@
     <col min="26" max="26" width="22.83203125" customWidth="1"/>
     <col min="27" max="27" width="22.83203125" customWidth="1"/>
     <col min="28" max="28" width="22.83203125" customWidth="1"/>
+    <col min="29" max="29" width="22.83203125" customWidth="1"/>
+    <col min="30" max="30" width="22.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
+        <v>issueDate</v>
+      </c>
+      <c r="B1" t="str">
         <v>fullNameAr</v>
       </c>
-      <c r="B1" t="str">
+      <c r="C1" t="str">
         <v>fullNameEn</v>
       </c>
-      <c r="C1" t="str">
+      <c r="D1" t="str">
         <v>surnameAr</v>
       </c>
-      <c r="D1" t="str">
+      <c r="E1" t="str">
         <v>surnameEn</v>
       </c>
-      <c r="E1" t="str">
+      <c r="F1" t="str">
+        <v>birthDate</v>
+      </c>
+      <c r="G1" t="str">
         <v>birthPlaceAr</v>
       </c>
-      <c r="F1" t="str">
+      <c r="H1" t="str">
         <v>birthPlaceEn</v>
       </c>
-      <c r="G1" t="str">
-        <v>birthDate</v>
-      </c>
-      <c r="H1" t="str">
+      <c r="I1" t="str">
+        <v>nationalityAr</v>
+      </c>
+      <c r="J1" t="str">
+        <v>nationalityEn</v>
+      </c>
+      <c r="K1" t="str">
         <v>idTypeAr</v>
       </c>
-      <c r="I1" t="str">
+      <c r="L1" t="str">
         <v>idTypeEn</v>
       </c>
-      <c r="J1" t="str">
+      <c r="M1" t="str">
         <v>idNumberAr</v>
       </c>
-      <c r="K1" t="str">
+      <c r="N1" t="str">
         <v>idNumberEn</v>
       </c>
-      <c r="L1" t="str">
+      <c r="O1" t="str">
+        <v>passportNoAr</v>
+      </c>
+      <c r="P1" t="str">
+        <v>passportNoEn</v>
+      </c>
+      <c r="Q1" t="str">
         <v>passportAr</v>
       </c>
-      <c r="M1" t="str">
+      <c r="R1" t="str">
         <v>passportEn</v>
       </c>
-      <c r="N1" t="str">
-        <v>nationalityAr</v>
-      </c>
-      <c r="O1" t="str">
-        <v>nationalityEn</v>
-      </c>
-      <c r="P1" t="str">
+      <c r="S1" t="str">
         <v>occupationAr</v>
       </c>
-      <c r="Q1" t="str">
+      <c r="T1" t="str">
         <v>occupationEn</v>
       </c>
-      <c r="R1" t="str">
+      <c r="U1" t="str">
         <v>idIssueDateAr</v>
       </c>
-      <c r="S1" t="str">
+      <c r="V1" t="str">
         <v>idIssueDateEn</v>
       </c>
-      <c r="T1" t="str">
+      <c r="W1" t="str">
         <v>idIssuePlaceAr</v>
       </c>
-      <c r="U1" t="str">
+      <c r="X1" t="str">
         <v>idIssuePlaceEn</v>
       </c>
-      <c r="V1" t="str">
+      <c r="Y1" t="str">
         <v>departmentAr</v>
       </c>
-      <c r="W1" t="str">
+      <c r="Z1" t="str">
         <v>departmentEn</v>
       </c>
-      <c r="X1" t="str">
-        <v>issueDate</v>
-      </c>
-      <c r="Y1" t="str">
+      <c r="AA1" t="str">
         <v>expiryAr</v>
       </c>
-      <c r="Z1" t="str">
+      <c r="AB1" t="str">
         <v>expiryEn</v>
       </c>
-      <c r="AA1" t="str">
+      <c r="AC1" t="str">
         <v>notesAr</v>
       </c>
-      <c r="AB1" t="str">
+      <c r="AD1" t="str">
         <v>notesEn</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
+        <v>11/12/2025</v>
+      </c>
+      <c r="B2" t="str">
         <v>جميل جبر أحمد</v>
       </c>
-      <c r="B2" t="str">
+      <c r="C2" t="str">
         <v>Jameel Jabr Ahmed</v>
       </c>
-      <c r="C2" t="str">
+      <c r="D2" t="str">
         <v>الرملي</v>
       </c>
-      <c r="D2" t="str">
+      <c r="E2" t="str">
         <v>Al Ramli</v>
       </c>
-      <c r="E2" t="str">
+      <c r="F2" t="str">
+        <v>16/02/1995</v>
+      </c>
+      <c r="G2" t="str">
         <v>السعودية، جدة</v>
       </c>
-      <c r="F2" t="str">
+      <c r="H2" t="str">
         <v>Jeddah, Saudi Arabia</v>
       </c>
-      <c r="G2" t="str">
-        <v>16/02/1995</v>
-      </c>
-      <c r="H2" t="str">
+      <c r="I2" t="str">
+        <v>اليمن</v>
+      </c>
+      <c r="J2" t="str">
+        <v>Yemen</v>
+      </c>
+      <c r="K2" t="str">
         <v>جواز سفر</v>
       </c>
-      <c r="I2" t="str">
+      <c r="L2" t="str">
         <v>Passport</v>
       </c>
-      <c r="J2" t="str">
+      <c r="M2" t="str">
         <v>10878313</v>
       </c>
-      <c r="K2" t="str">
+      <c r="N2" t="str">
         <v>10878313</v>
       </c>
-      <c r="L2" t="str">
+      <c r="O2" t="str">
+        <v>P0000000</v>
+      </c>
+      <c r="P2" t="str">
+        <v>P0000000</v>
+      </c>
+      <c r="Q2" t="str">
         <v>11/03/2026</v>
       </c>
-      <c r="M2" t="str">
+      <c r="R2" t="str">
         <v>11/03/2026</v>
       </c>
-      <c r="N2" t="str">
-        <v>اليمن</v>
-      </c>
-      <c r="O2" t="str">
-        <v>Yemen</v>
-      </c>
-      <c r="P2" t="str">
+      <c r="S2" t="str">
         <v>منسوب مبيعات</v>
       </c>
-      <c r="Q2" t="str">
+      <c r="T2" t="str">
         <v>Sales Representative</v>
       </c>
-      <c r="R2" t="str">
+      <c r="U2" t="str">
         <v>01/03/2023</v>
       </c>
-      <c r="S2" t="str">
+      <c r="V2" t="str">
         <v>01/03/2023</v>
       </c>
-      <c r="T2" t="str">
+      <c r="W2" t="str">
         <v>معين</v>
       </c>
-      <c r="U2" t="str">
+      <c r="X2" t="str">
         <v>Ma'in</v>
       </c>
-      <c r="V2" t="str">
+      <c r="Y2" t="str">
         <v>سفارة عمان</v>
       </c>
-      <c r="W2" t="str">
+      <c r="Z2" t="str">
         <v>Embassy of Oman</v>
       </c>
-      <c r="X2" t="str">
-        <v>11/12/2025</v>
-      </c>
-      <c r="Y2" t="str">
+      <c r="AA2" t="str">
         <v>11/03/2026</v>
       </c>
-      <c r="Z2" t="str">
+      <c r="AB2" t="str">
         <v>11/03/2026</v>
       </c>
-      <c r="AA2" t="str">
+      <c r="AC2" t="str">
         <v>تم التحقق من سجلاتنا.</v>
       </c>
-      <c r="AB2" t="str">
+      <c r="AD2" t="str">
         <v>OUR RECORDS HAVE BEEN VERIFIED.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AD2"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:A9"/>
+  <dimension ref="A1:A6"/>
   <cols>
     <col min="1" max="1" width="120.83203125" customWidth="1"/>
   </cols>
@@ -633,7 +648,7 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>الأرقام النظامية ينشئها النظام تلقائيًا ولا تُستورد من Excel.</v>
+        <v>الأرقام النظامية issueNo و referenceNo و internalNo و issuanceNo لا تكتبها؛ ينشئها النظام بعد الاستيراد.</v>
       </c>
     </row>
     <row r="5">
@@ -643,27 +658,477 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>مقاس الصورة الموصى به: 400 × 600 بكسل بنسبة 2:3، JPG أو PNG، وبحد أقصى 5MB.</v>
+        <v>لا تغيّر أسماء أعمدة ورقة Good Conduct حتى يتم الاستيراد بشكل صحيح.</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:A6"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:D32"/>
+  <cols>
+    <col min="1" max="1" width="34.83203125" customWidth="1"/>
+    <col min="2" max="2" width="32.83203125" customWidth="1"/>
+    <col min="3" max="3" width="34.83203125" customWidth="1"/>
+    <col min="4" max="4" width="42.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>اسم الحقل الداخلي</v>
+      </c>
+      <c r="B1" t="str">
+        <v>التسمية العربية</v>
+      </c>
+      <c r="C1" t="str">
+        <v>التسمية الإنجليزية</v>
+      </c>
+      <c r="D1" t="str">
+        <v>ملاحظة</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>issueDate</v>
+      </c>
+      <c r="B2" t="str">
+        <v>تاريخ الإصدار</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Issue Date</v>
+      </c>
+      <c r="D2" t="str">
+        <v>بيانات مستخدم قابلة للاستيراد</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>fullNameAr</v>
+      </c>
+      <c r="B3" t="str">
+        <v>الاسم الكامل</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Full Name</v>
+      </c>
+      <c r="D3" t="str">
+        <v>بيانات مستخدم قابلة للاستيراد</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>fullNameEn</v>
+      </c>
+      <c r="B4" t="str">
+        <v>الاسم بالإنجليزي</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Full Name (English)</v>
+      </c>
+      <c r="D4" t="str">
+        <v>بيانات مستخدم قابلة للاستيراد</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>surnameAr</v>
+      </c>
+      <c r="B5" t="str">
+        <v>اللقب</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Surname</v>
+      </c>
+      <c r="D5" t="str">
+        <v>بيانات مستخدم قابلة للاستيراد</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>surnameEn</v>
+      </c>
+      <c r="B6" t="str">
+        <v>اللقب بالإنجليزي</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Surname (English)</v>
+      </c>
+      <c r="D6" t="str">
+        <v>بيانات مستخدم قابلة للاستيراد</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>تُستخدم الصورة نفسها للعلامة المائية، ويزيل النظام الخلفية البيضاء من نسختها فقط.</v>
+        <v>birthDate</v>
+      </c>
+      <c r="B7" t="str">
+        <v>تاريخ الميلاد</v>
+      </c>
+      <c r="C7" t="str">
+        <v>Birth Date</v>
+      </c>
+      <c r="D7" t="str">
+        <v>بيانات مستخدم قابلة للاستيراد</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>مقاس الصورة داخل الوثيقة: 40 × 60mm. مقاس العلامة المائية: 24 × 36mm تقريبًا.</v>
+        <v>birthPlaceAr</v>
+      </c>
+      <c r="B8" t="str">
+        <v>مكان الميلاد</v>
+      </c>
+      <c r="C8" t="str">
+        <v>Birth Place</v>
+      </c>
+      <c r="D8" t="str">
+        <v>بيانات مستخدم قابلة للاستيراد</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>لا تغيّر أسماء أعمدة ورقة Good Conduct حتى يتم الاستيراد بشكل صحيح.</v>
+        <v>birthPlaceEn</v>
+      </c>
+      <c r="B9" t="str">
+        <v>مكان الميلاد بالإنجليزي</v>
+      </c>
+      <c r="C9" t="str">
+        <v>Birth Place (English)</v>
+      </c>
+      <c r="D9" t="str">
+        <v>بيانات مستخدم قابلة للاستيراد</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>nationalityAr</v>
+      </c>
+      <c r="B10" t="str">
+        <v>الجنسية</v>
+      </c>
+      <c r="C10" t="str">
+        <v>Nationality</v>
+      </c>
+      <c r="D10" t="str">
+        <v>بيانات مستخدم قابلة للاستيراد</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>nationalityEn</v>
+      </c>
+      <c r="B11" t="str">
+        <v>الجنسية بالإنجليزي</v>
+      </c>
+      <c r="C11" t="str">
+        <v>Nationality (English)</v>
+      </c>
+      <c r="D11" t="str">
+        <v>بيانات مستخدم قابلة للاستيراد</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>idTypeAr</v>
+      </c>
+      <c r="B12" t="str">
+        <v>نوع الهوية</v>
+      </c>
+      <c r="C12" t="str">
+        <v>ID Type</v>
+      </c>
+      <c r="D12" t="str">
+        <v>بيانات مستخدم قابلة للاستيراد</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>idTypeEn</v>
+      </c>
+      <c r="B13" t="str">
+        <v>نوع الهوية بالإنجليزي</v>
+      </c>
+      <c r="C13" t="str">
+        <v>ID Type (English)</v>
+      </c>
+      <c r="D13" t="str">
+        <v>بيانات مستخدم قابلة للاستيراد</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>idNumberAr</v>
+      </c>
+      <c r="B14" t="str">
+        <v>رقم الهوية</v>
+      </c>
+      <c r="C14" t="str">
+        <v>ID Number</v>
+      </c>
+      <c r="D14" t="str">
+        <v>بيانات مستخدم قابلة للاستيراد</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>idNumberEn</v>
+      </c>
+      <c r="B15" t="str">
+        <v>رقم الهوية بالإنجليزي</v>
+      </c>
+      <c r="C15" t="str">
+        <v>ID Number (English)</v>
+      </c>
+      <c r="D15" t="str">
+        <v>بيانات مستخدم قابلة للاستيراد</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>passportNoAr</v>
+      </c>
+      <c r="B16" t="str">
+        <v>رقم الجواز</v>
+      </c>
+      <c r="C16" t="str">
+        <v>Passport Number</v>
+      </c>
+      <c r="D16" t="str">
+        <v>بيانات مستخدم قابلة للاستيراد</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>passportNoEn</v>
+      </c>
+      <c r="B17" t="str">
+        <v>رقم الجواز بالإنجليزي</v>
+      </c>
+      <c r="C17" t="str">
+        <v>Passport Number (English)</v>
+      </c>
+      <c r="D17" t="str">
+        <v>بيانات مستخدم قابلة للاستيراد</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>passportAr</v>
+      </c>
+      <c r="B18" t="str">
+        <v>تاريخ انتهاء الجواز</v>
+      </c>
+      <c r="C18" t="str">
+        <v>Passport Expiry</v>
+      </c>
+      <c r="D18" t="str">
+        <v>بيانات مستخدم قابلة للاستيراد</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>passportEn</v>
+      </c>
+      <c r="B19" t="str">
+        <v>تاريخ انتهاء الجواز بالإنجليزي</v>
+      </c>
+      <c r="C19" t="str">
+        <v>Passport Expiry (English)</v>
+      </c>
+      <c r="D19" t="str">
+        <v>بيانات مستخدم قابلة للاستيراد</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>occupationAr</v>
+      </c>
+      <c r="B20" t="str">
+        <v>المهنة</v>
+      </c>
+      <c r="C20" t="str">
+        <v>Occupation</v>
+      </c>
+      <c r="D20" t="str">
+        <v>بيانات مستخدم قابلة للاستيراد</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>occupationEn</v>
+      </c>
+      <c r="B21" t="str">
+        <v>المهنة بالإنجليزي</v>
+      </c>
+      <c r="C21" t="str">
+        <v>Occupation (English)</v>
+      </c>
+      <c r="D21" t="str">
+        <v>بيانات مستخدم قابلة للاستيراد</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>idIssueDateAr</v>
+      </c>
+      <c r="B22" t="str">
+        <v>تاريخ إصدار الهوية</v>
+      </c>
+      <c r="C22" t="str">
+        <v>ID Issue Date</v>
+      </c>
+      <c r="D22" t="str">
+        <v>بيانات مستخدم قابلة للاستيراد</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>idIssueDateEn</v>
+      </c>
+      <c r="B23" t="str">
+        <v>تاريخ إصدار الهوية بالإنجليزي</v>
+      </c>
+      <c r="C23" t="str">
+        <v>ID Issue Date (English)</v>
+      </c>
+      <c r="D23" t="str">
+        <v>بيانات مستخدم قابلة للاستيراد</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>idIssuePlaceAr</v>
+      </c>
+      <c r="B24" t="str">
+        <v>جهة إصدار الهوية</v>
+      </c>
+      <c r="C24" t="str">
+        <v>ID Issue Place</v>
+      </c>
+      <c r="D24" t="str">
+        <v>بيانات مستخدم قابلة للاستيراد</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>idIssuePlaceEn</v>
+      </c>
+      <c r="B25" t="str">
+        <v>جهة إصدار الهوية بالإنجليزي</v>
+      </c>
+      <c r="C25" t="str">
+        <v>ID Issue Place (English)</v>
+      </c>
+      <c r="D25" t="str">
+        <v>بيانات مستخدم قابلة للاستيراد</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>departmentAr</v>
+      </c>
+      <c r="B26" t="str">
+        <v>الجهة التي سيُقدَّم إليها</v>
+      </c>
+      <c r="C26" t="str">
+        <v>Department Requested</v>
+      </c>
+      <c r="D26" t="str">
+        <v>بيانات مستخدم قابلة للاستيراد</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>departmentEn</v>
+      </c>
+      <c r="B27" t="str">
+        <v>الجهة التي سيُقدَّم إليها بالإنجليزي</v>
+      </c>
+      <c r="C27" t="str">
+        <v>Department Requested (English)</v>
+      </c>
+      <c r="D27" t="str">
+        <v>بيانات مستخدم قابلة للاستيراد</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>expiryAr</v>
+      </c>
+      <c r="B28" t="str">
+        <v>تاريخ انتهاء الوثيقة</v>
+      </c>
+      <c r="C28" t="str">
+        <v>Document Expiry</v>
+      </c>
+      <c r="D28" t="str">
+        <v>بيانات مستخدم قابلة للاستيراد</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v>expiryEn</v>
+      </c>
+      <c r="B29" t="str">
+        <v>تاريخ انتهاء الوثيقة بالإنجليزي</v>
+      </c>
+      <c r="C29" t="str">
+        <v>Document Expiry (English)</v>
+      </c>
+      <c r="D29" t="str">
+        <v>بيانات مستخدم قابلة للاستيراد</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v>notesAr</v>
+      </c>
+      <c r="B30" t="str">
+        <v>الملاحظة</v>
+      </c>
+      <c r="C30" t="str">
+        <v>Notes</v>
+      </c>
+      <c r="D30" t="str">
+        <v>بيانات مستخدم قابلة للاستيراد</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="str">
+        <v>notesEn</v>
+      </c>
+      <c r="B31" t="str">
+        <v>الملاحظة بالإنجليزي</v>
+      </c>
+      <c r="C31" t="str">
+        <v>Notes (English)</v>
+      </c>
+      <c r="D31" t="str">
+        <v>بيانات مستخدم قابلة للاستيراد</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="str">
+        <v>issueNo / referenceNo / internalNo / issuanceNo</v>
+      </c>
+      <c r="B32" t="str">
+        <v>أرقام النظام</v>
+      </c>
+      <c r="C32" t="str">
+        <v>System identifiers</v>
+      </c>
+      <c r="D32" t="str">
+        <v>لا تعبئها؛ ينشئها النظام بعد الاستيراد</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:A9"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D32"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix: publish page identity links and printable barcode
</commit_message>
<xml_diff>
--- a/Good Conduct Data Template.xlsx
+++ b/Good Conduct Data Template.xlsx
@@ -399,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AD2"/>
+  <dimension ref="A1:AB2"/>
   <cols>
     <col min="1" max="1" width="22.83203125" customWidth="1"/>
     <col min="2" max="2" width="22.83203125" customWidth="1"/>
@@ -429,8 +429,6 @@
     <col min="26" max="26" width="22.83203125" customWidth="1"/>
     <col min="27" max="27" width="22.83203125" customWidth="1"/>
     <col min="28" max="28" width="22.83203125" customWidth="1"/>
-    <col min="29" max="29" width="22.83203125" customWidth="1"/>
-    <col min="30" max="30" width="22.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -477,51 +475,45 @@
         <v>idNumberEn</v>
       </c>
       <c r="O1" t="str">
-        <v>passportNoAr</v>
+        <v>passportAr</v>
       </c>
       <c r="P1" t="str">
-        <v>passportNoEn</v>
+        <v>passportEn</v>
       </c>
       <c r="Q1" t="str">
-        <v>passportAr</v>
+        <v>occupationAr</v>
       </c>
       <c r="R1" t="str">
-        <v>passportEn</v>
+        <v>occupationEn</v>
       </c>
       <c r="S1" t="str">
-        <v>occupationAr</v>
+        <v>idIssueDateAr</v>
       </c>
       <c r="T1" t="str">
-        <v>occupationEn</v>
+        <v>idIssueDateEn</v>
       </c>
       <c r="U1" t="str">
-        <v>idIssueDateAr</v>
+        <v>idIssuePlaceAr</v>
       </c>
       <c r="V1" t="str">
-        <v>idIssueDateEn</v>
+        <v>idIssuePlaceEn</v>
       </c>
       <c r="W1" t="str">
-        <v>idIssuePlaceAr</v>
+        <v>departmentAr</v>
       </c>
       <c r="X1" t="str">
-        <v>idIssuePlaceEn</v>
+        <v>departmentEn</v>
       </c>
       <c r="Y1" t="str">
-        <v>departmentAr</v>
+        <v>expiryAr</v>
       </c>
       <c r="Z1" t="str">
-        <v>departmentEn</v>
+        <v>expiryEn</v>
       </c>
       <c r="AA1" t="str">
-        <v>expiryAr</v>
+        <v>notesAr</v>
       </c>
       <c r="AB1" t="str">
-        <v>expiryEn</v>
-      </c>
-      <c r="AC1" t="str">
-        <v>notesAr</v>
-      </c>
-      <c r="AD1" t="str">
         <v>notesEn</v>
       </c>
     </row>
@@ -569,57 +561,51 @@
         <v>10878313</v>
       </c>
       <c r="O2" t="str">
-        <v>P0000000</v>
+        <v>11/03/2026</v>
       </c>
       <c r="P2" t="str">
-        <v>P0000000</v>
+        <v>11/03/2026</v>
       </c>
       <c r="Q2" t="str">
+        <v>منسوب مبيعات</v>
+      </c>
+      <c r="R2" t="str">
+        <v>Sales Representative</v>
+      </c>
+      <c r="S2" t="str">
+        <v>01/03/2023</v>
+      </c>
+      <c r="T2" t="str">
+        <v>01/03/2023</v>
+      </c>
+      <c r="U2" t="str">
+        <v>معين</v>
+      </c>
+      <c r="V2" t="str">
+        <v>Ma'in</v>
+      </c>
+      <c r="W2" t="str">
+        <v>سفارة عمان</v>
+      </c>
+      <c r="X2" t="str">
+        <v>Embassy of Oman</v>
+      </c>
+      <c r="Y2" t="str">
         <v>11/03/2026</v>
       </c>
-      <c r="R2" t="str">
+      <c r="Z2" t="str">
         <v>11/03/2026</v>
       </c>
-      <c r="S2" t="str">
-        <v>منسوب مبيعات</v>
-      </c>
-      <c r="T2" t="str">
-        <v>Sales Representative</v>
-      </c>
-      <c r="U2" t="str">
-        <v>01/03/2023</v>
-      </c>
-      <c r="V2" t="str">
-        <v>01/03/2023</v>
-      </c>
-      <c r="W2" t="str">
-        <v>معين</v>
-      </c>
-      <c r="X2" t="str">
-        <v>Ma'in</v>
-      </c>
-      <c r="Y2" t="str">
-        <v>سفارة عمان</v>
-      </c>
-      <c r="Z2" t="str">
-        <v>Embassy of Oman</v>
-      </c>
       <c r="AA2" t="str">
-        <v>11/03/2026</v>
+        <v>تم التحقق من سجلاتنا.</v>
       </c>
       <c r="AB2" t="str">
-        <v>11/03/2026</v>
-      </c>
-      <c r="AC2" t="str">
-        <v>تم التحقق من سجلاتنا.</v>
-      </c>
-      <c r="AD2" t="str">
         <v>OUR RECORDS HAVE BEEN VERIFIED.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AD2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB2"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -670,7 +656,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D32"/>
+  <dimension ref="A1:D30"/>
   <cols>
     <col min="1" max="1" width="34.83203125" customWidth="1"/>
     <col min="2" max="2" width="32.83203125" customWidth="1"/>
@@ -890,13 +876,13 @@
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>passportNoAr</v>
+        <v>passportAr</v>
       </c>
       <c r="B16" t="str">
-        <v>رقم الجواز</v>
+        <v>تاريخ انتهاء الجواز</v>
       </c>
       <c r="C16" t="str">
-        <v>Passport Number</v>
+        <v>Passport Expiry</v>
       </c>
       <c r="D16" t="str">
         <v>بيانات مستخدم قابلة للاستيراد</v>
@@ -904,13 +890,13 @@
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>passportNoEn</v>
+        <v>passportEn</v>
       </c>
       <c r="B17" t="str">
-        <v>رقم الجواز بالإنجليزي</v>
+        <v>تاريخ انتهاء الجواز بالإنجليزي</v>
       </c>
       <c r="C17" t="str">
-        <v>Passport Number (English)</v>
+        <v>Passport Expiry (English)</v>
       </c>
       <c r="D17" t="str">
         <v>بيانات مستخدم قابلة للاستيراد</v>
@@ -918,13 +904,13 @@
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>passportAr</v>
+        <v>occupationAr</v>
       </c>
       <c r="B18" t="str">
-        <v>تاريخ انتهاء الجواز</v>
+        <v>المهنة</v>
       </c>
       <c r="C18" t="str">
-        <v>Passport Expiry</v>
+        <v>Occupation</v>
       </c>
       <c r="D18" t="str">
         <v>بيانات مستخدم قابلة للاستيراد</v>
@@ -932,13 +918,13 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>passportEn</v>
+        <v>occupationEn</v>
       </c>
       <c r="B19" t="str">
-        <v>تاريخ انتهاء الجواز بالإنجليزي</v>
+        <v>المهنة بالإنجليزي</v>
       </c>
       <c r="C19" t="str">
-        <v>Passport Expiry (English)</v>
+        <v>Occupation (English)</v>
       </c>
       <c r="D19" t="str">
         <v>بيانات مستخدم قابلة للاستيراد</v>
@@ -946,13 +932,13 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>occupationAr</v>
+        <v>idIssueDateAr</v>
       </c>
       <c r="B20" t="str">
-        <v>المهنة</v>
+        <v>تاريخ إصدار الهوية</v>
       </c>
       <c r="C20" t="str">
-        <v>Occupation</v>
+        <v>ID Issue Date</v>
       </c>
       <c r="D20" t="str">
         <v>بيانات مستخدم قابلة للاستيراد</v>
@@ -960,13 +946,13 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>occupationEn</v>
+        <v>idIssueDateEn</v>
       </c>
       <c r="B21" t="str">
-        <v>المهنة بالإنجليزي</v>
+        <v>تاريخ إصدار الهوية بالإنجليزي</v>
       </c>
       <c r="C21" t="str">
-        <v>Occupation (English)</v>
+        <v>ID Issue Date (English)</v>
       </c>
       <c r="D21" t="str">
         <v>بيانات مستخدم قابلة للاستيراد</v>
@@ -974,13 +960,13 @@
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>idIssueDateAr</v>
+        <v>idIssuePlaceAr</v>
       </c>
       <c r="B22" t="str">
-        <v>تاريخ إصدار الهوية</v>
+        <v>جهة إصدار الهوية</v>
       </c>
       <c r="C22" t="str">
-        <v>ID Issue Date</v>
+        <v>ID Issue Place</v>
       </c>
       <c r="D22" t="str">
         <v>بيانات مستخدم قابلة للاستيراد</v>
@@ -988,13 +974,13 @@
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>idIssueDateEn</v>
+        <v>idIssuePlaceEn</v>
       </c>
       <c r="B23" t="str">
-        <v>تاريخ إصدار الهوية بالإنجليزي</v>
+        <v>جهة إصدار الهوية بالإنجليزي</v>
       </c>
       <c r="C23" t="str">
-        <v>ID Issue Date (English)</v>
+        <v>ID Issue Place (English)</v>
       </c>
       <c r="D23" t="str">
         <v>بيانات مستخدم قابلة للاستيراد</v>
@@ -1002,13 +988,13 @@
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>idIssuePlaceAr</v>
+        <v>departmentAr</v>
       </c>
       <c r="B24" t="str">
-        <v>جهة إصدار الهوية</v>
+        <v>الجهة التي سيُقدَّم إليها</v>
       </c>
       <c r="C24" t="str">
-        <v>ID Issue Place</v>
+        <v>Department Requested</v>
       </c>
       <c r="D24" t="str">
         <v>بيانات مستخدم قابلة للاستيراد</v>
@@ -1016,13 +1002,13 @@
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>idIssuePlaceEn</v>
+        <v>departmentEn</v>
       </c>
       <c r="B25" t="str">
-        <v>جهة إصدار الهوية بالإنجليزي</v>
+        <v>الجهة التي سيُقدَّم إليها بالإنجليزي</v>
       </c>
       <c r="C25" t="str">
-        <v>ID Issue Place (English)</v>
+        <v>Department Requested (English)</v>
       </c>
       <c r="D25" t="str">
         <v>بيانات مستخدم قابلة للاستيراد</v>
@@ -1030,13 +1016,13 @@
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>departmentAr</v>
+        <v>expiryAr</v>
       </c>
       <c r="B26" t="str">
-        <v>الجهة التي سيُقدَّم إليها</v>
+        <v>تاريخ انتهاء الوثيقة</v>
       </c>
       <c r="C26" t="str">
-        <v>Department Requested</v>
+        <v>Document Expiry</v>
       </c>
       <c r="D26" t="str">
         <v>بيانات مستخدم قابلة للاستيراد</v>
@@ -1044,13 +1030,13 @@
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>departmentEn</v>
+        <v>expiryEn</v>
       </c>
       <c r="B27" t="str">
-        <v>الجهة التي سيُقدَّم إليها بالإنجليزي</v>
+        <v>تاريخ انتهاء الوثيقة بالإنجليزي</v>
       </c>
       <c r="C27" t="str">
-        <v>Department Requested (English)</v>
+        <v>Document Expiry (English)</v>
       </c>
       <c r="D27" t="str">
         <v>بيانات مستخدم قابلة للاستيراد</v>
@@ -1058,13 +1044,13 @@
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>expiryAr</v>
+        <v>notesAr</v>
       </c>
       <c r="B28" t="str">
-        <v>تاريخ انتهاء الوثيقة</v>
+        <v>الملاحظة</v>
       </c>
       <c r="C28" t="str">
-        <v>Document Expiry</v>
+        <v>Notes</v>
       </c>
       <c r="D28" t="str">
         <v>بيانات مستخدم قابلة للاستيراد</v>
@@ -1072,13 +1058,13 @@
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>expiryEn</v>
+        <v>notesEn</v>
       </c>
       <c r="B29" t="str">
-        <v>تاريخ انتهاء الوثيقة بالإنجليزي</v>
+        <v>الملاحظة بالإنجليزي</v>
       </c>
       <c r="C29" t="str">
-        <v>Document Expiry (English)</v>
+        <v>Notes (English)</v>
       </c>
       <c r="D29" t="str">
         <v>بيانات مستخدم قابلة للاستيراد</v>
@@ -1086,49 +1072,21 @@
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>notesAr</v>
+        <v>issueNo / referenceNo / internalNo / issuanceNo</v>
       </c>
       <c r="B30" t="str">
-        <v>الملاحظة</v>
+        <v>أرقام النظام</v>
       </c>
       <c r="C30" t="str">
-        <v>Notes</v>
+        <v>System identifiers</v>
       </c>
       <c r="D30" t="str">
-        <v>بيانات مستخدم قابلة للاستيراد</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="str">
-        <v>notesEn</v>
-      </c>
-      <c r="B31" t="str">
-        <v>الملاحظة بالإنجليزي</v>
-      </c>
-      <c r="C31" t="str">
-        <v>Notes (English)</v>
-      </c>
-      <c r="D31" t="str">
-        <v>بيانات مستخدم قابلة للاستيراد</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="str">
-        <v>issueNo / referenceNo / internalNo / issuanceNo</v>
-      </c>
-      <c r="B32" t="str">
-        <v>أرقام النظام</v>
-      </c>
-      <c r="C32" t="str">
-        <v>System identifiers</v>
-      </c>
-      <c r="D32" t="str">
         <v>لا تعبئها؛ ينشئها النظام بعد الاستيراد</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D32"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D30"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>